<commit_message>
Translate skill docs, templates and example to English
Template labels are now English and rendered in the document language
(Thai by default); README rewritten in English with install steps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiLF94QhvD1XTnDF8RiZLC
</commit_message>
<xml_diff>
--- a/docs/examples/TC_SALES_v18_20261013.xlsx
+++ b/docs/examples/TC_SALES_v18_20261013.xlsx
@@ -526,7 +526,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -597,7 +597,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>สร้างใบเสนอราคาและยืนยัน</t>
+          <t>Create and confirm quotation</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -613,7 +613,7 @@
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>1. Sales &gt; Orders &gt; Quotations &gt; New
-2. เลือก Customer, เพิ่ม Product
+2. Select Customer, add Product
 3. Confirm</t>
         </is>
       </c>
@@ -624,7 +624,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>State = Sales Order; Delivery 1 ใบ; Untaxed 2,000 / Tax 140 / Total 2,140</t>
+          <t>State = Sales Order; 1 Delivery created; Untaxed 2,000 / Tax 140 / Total 2,140</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ไม่ระบุลูกค้า</t>
+          <t>Save without customer</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>1. New
-2. ไม่เลือก Customer กด Save</t>
+2. Leave Customer empty, click Save</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>แสดง error ฟิลด์ Customer บังคับ, บันทึกไม่ได้</t>
+          <t>Error: Customer is required; record not saved</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ออก Invoice ก่อนส่งของ</t>
+          <t>Invoice before delivery</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1. เปิด SO
+          <t>1. Open SO
 2. Create Invoice</t>
         </is>
       </c>
@@ -722,7 +722,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>แจ้งไม่มีรายการให้ออก Invoice (Delivered = 0)</t>
+          <t>Message: nothing to invoice (Delivered = 0)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -749,7 +749,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ส่งของบางส่วน + Backorder</t>
+          <t>Partial delivery + backorder</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>DO Done 1, Backorder 1 ชิ้น, On Hand 9</t>
+          <t>DO Done 1, Backorder 1 unit, On Hand 9</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ออก Invoice ตามที่ส่ง</t>
+          <t>Invoice delivered quantity</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>จำนวน 0</t>
+          <t>Zero quantity</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1. New เพิ่ม P001 qty 0
+          <t>1. New, add P001 qty 0
 2. Confirm</t>
         </is>
       </c>
@@ -874,7 +874,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ไม่สร้าง Delivery / ไม่มียอด (verify behaviour ที่ลูกค้าต้องการ)</t>
+          <t>No Delivery created, amount 0 (verify behavior the customer expects)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">

</xml_diff>